<commit_message>
Fix UnboundLocalError by removing redundant import re
</commit_message>
<xml_diff>
--- a/output/classified_messages.xlsx
+++ b/output/classified_messages.xlsx
@@ -453,7 +453,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>BREAKING: Water levels in Kelani River (Colombo) h</t>
+          <t>BREAKING: Water levels in Kelani River (Colombo) h...</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -463,19 +463,19 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Info</t>
+          <t>Supply</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Low</t>
+          <t>Medium</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>SOS: 5 people trapped on a roof in Ja-Ela (Gampaha</t>
+          <t>SOS: 5 people trapped on a roof in Ja-Ela (Gampaha...</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -497,17 +497,17 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Update: Kandy road cleared near Peradeniya. Traffi</t>
+          <t>Update: Kandy road cleared near Peradeniya. Traffi...</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Unknown</t>
+          <t>Kandy</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Other</t>
+          <t>Info</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
@@ -519,7 +519,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Does anyone have extra dry rations for the camp in</t>
+          <t>Does anyone have extra dry rations for the camp in...</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -551,12 +551,12 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Other</t>
+          <t>Supply</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Low</t>
+          <t>Medium</t>
         </is>
       </c>
     </row>
@@ -573,7 +573,7 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Other</t>
+          <t>Info</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
@@ -585,34 +585,34 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Just saw on news that Gampaha town is flooded. Hop</t>
+          <t>Just saw on news that Gampaha town is flooded. Hop...</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Unknown</t>
+          <t>Gampaha</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Other</t>
+          <t>Info</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Low</t>
+          <t>Medium</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>We are trapped in the attic. 3 kids. Water is ente</t>
+          <t>We are trapped in the attic. 3 kids. Water is ente...</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Gampaha</t>
+          <t>Unknown</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -629,7 +629,7 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Donation drive happening at the town hall tomorrow</t>
+          <t>Donation drive happening at the town hall tomorrow...</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -639,19 +639,19 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Other</t>
+          <t>Supply</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>Low</t>
+          <t>Medium</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Report: Heavy rains expected to continue for the n</t>
+          <t>Report: Heavy rains expected to continue for the n...</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -661,24 +661,24 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Other</t>
+          <t>Info</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>Low</t>
+          <t>Medium</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>URGENT: Landslide in Badulla. 2 houses buried. Nee</t>
+          <t>URGENT: Landslide in Badulla. 2 houses buried. Nee...</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Kalutara</t>
+          <t>Unknown</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
@@ -705,7 +705,7 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Other</t>
+          <t>Info</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
@@ -717,7 +717,7 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>The Navy has deployed 5 boats to the Kelaniya area</t>
+          <t>The Navy has deployed 5 boats to the Kelaniya area...</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -727,7 +727,7 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Other</t>
+          <t>Info</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
@@ -739,12 +739,12 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Help! My grandmother is bedridden and the water is</t>
+          <t>Help! My grandmother is bedridden and the water is...</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Gampaha</t>
+          <t>Unknown</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -771,7 +771,7 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Other</t>
+          <t>Info</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
@@ -783,34 +783,34 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t xml:space="preserve">Gampaha hospital is requesting drinking water for </t>
+          <t>Gampaha hospital is requesting drinking water for ...</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Unknown</t>
+          <t>Gampaha</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Other</t>
+          <t>Supply</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>Low</t>
+          <t>Medium</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>SOS: 10 people stranded on a rock in Kitulgala. Wa</t>
+          <t>SOS: 10 people stranded on a rock in Kitulgala. Wa...</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Gampaha</t>
+          <t>Unknown</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
@@ -827,7 +827,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Just arrived at the shelter. It's crowded but safe</t>
+          <t>Just arrived at the shelter. It's crowded but safe...</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
@@ -837,7 +837,7 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Other</t>
+          <t>Info</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
@@ -849,7 +849,7 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Warning: Dengue risk is high due to stagnant water</t>
+          <t>Warning: Dengue risk is high due to stagnant water...</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
@@ -859,12 +859,12 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Other</t>
+          <t>Supply</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>Low</t>
+          <t>Medium</t>
         </is>
       </c>
     </row>
@@ -881,19 +881,19 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Other</t>
+          <t>Rescue</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>Low</t>
+          <t>High</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>My dog is missing in Kaduwela. Has anyone seen him</t>
+          <t>My dog is missing in Kaduwela. Has anyone seen him...</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
@@ -903,7 +903,7 @@
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>Other</t>
+          <t>Info</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
@@ -915,7 +915,7 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>The government has allocated 50 million rupees for</t>
+          <t>The government has allocated 50 million rupees for...</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
@@ -925,7 +925,7 @@
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Other</t>
+          <t>Info</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
@@ -937,7 +937,7 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>We need milk powder for 10 babies at the temple ca</t>
+          <t>We need milk powder for 10 babies at the temple ca...</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
@@ -947,7 +947,7 @@
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Other</t>
+          <t>Info</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
@@ -959,29 +959,29 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Colombo Fort station is dry. Trains are running on</t>
+          <t>Colombo Fort station is dry. Trains are running on...</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Unknown</t>
+          <t>Colombo</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>Other</t>
+          <t>Info</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>Low</t>
+          <t>Medium</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Emergency: Tree fell on a house in Wattala. 2 inju</t>
+          <t>Emergency: Tree fell on a house in Wattala. 2 inju...</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
@@ -991,12 +991,12 @@
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>Other</t>
+          <t>Rescue</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>Low</t>
+          <t>High</t>
         </is>
       </c>
     </row>
@@ -1008,12 +1008,12 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Unknown</t>
+          <t>Matara</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>Other</t>
+          <t>Info</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
@@ -1025,17 +1025,17 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>Kalutara bridge is at risk of collapse. Police hav</t>
+          <t>Kalutara bridge is at risk of collapse. Police hav...</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>Unknown</t>
+          <t>Kalutara</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>Other</t>
+          <t>Info</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
@@ -1047,22 +1047,22 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t xml:space="preserve">Rescue needed: Pregnant woman in labor at Ja-Ela. </t>
+          <t>Rescue needed: Pregnant woman in labor at Ja-Ela. ...</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>Unknown</t>
+          <t>Ja-Ela</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>Other</t>
+          <t>Rescue</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>Low</t>
+          <t>High</t>
         </is>
       </c>
     </row>
@@ -1074,12 +1074,12 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>Unknown</t>
+          <t>Galle</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>Other</t>
+          <t>Info</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
@@ -1091,29 +1091,29 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>River overflow in Ratnapura. Level 5.0m. Warning i</t>
+          <t>River overflow in Ratnapura. Level 5.0m. Warning i...</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Colombo</t>
+          <t>Unknown</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>Info</t>
+          <t>Rescue</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>Low</t>
+          <t>High</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>Wellampitiya is 100% underwater. 5000 people displ</t>
+          <t>Wellampitiya is 100% underwater. 5000 people displ...</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
@@ -1123,12 +1123,12 @@
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>Other</t>
+          <t>Supply</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>Low</t>
+          <t>Medium</t>
         </is>
       </c>
     </row>
@@ -1140,12 +1140,12 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>Unknown</t>
+          <t>Galle</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>Other</t>
+          <t>Info</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
@@ -1157,7 +1157,7 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>Donation needed: 500 packets of rice and curry for</t>
+          <t>Donation needed: 500 packets of rice and curry for...</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
@@ -1167,12 +1167,12 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>Other</t>
+          <t>Supply</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>Low</t>
+          <t>Medium</t>
         </is>
       </c>
     </row>
@@ -1189,34 +1189,34 @@
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>Other</t>
+          <t>Info</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>Low</t>
+          <t>Medium</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>SOS: Boat capsized in Gampaha. 3 people in the wat</t>
+          <t>SOS: Boat capsized in Gampaha. 3 people in the wat...</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>Unknown</t>
+          <t>Gampaha</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>Other</t>
+          <t>Rescue</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>Low</t>
+          <t>High</t>
         </is>
       </c>
     </row>
@@ -1233,29 +1233,29 @@
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>Other</t>
+          <t>Info</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>Low</t>
+          <t>Medium</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>Update: Electricity restored in some parts of Colo</t>
+          <t>Update: Electricity restored in some parts of Colo...</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>Unknown</t>
+          <t>Colombo</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>Other</t>
+          <t>Info</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
@@ -1277,7 +1277,7 @@
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>Other</t>
+          <t>Info</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
@@ -1289,12 +1289,12 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>Critical: Landslide warning issued for Kegalle dis</t>
+          <t>Critical: Landslide warning issued for Kegalle dis...</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>Kalutara</t>
+          <t>Galle</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
@@ -1311,7 +1311,7 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>Need volunteers to pack food parcels at the commun</t>
+          <t>Need volunteers to pack food parcels at the commun...</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
@@ -1321,34 +1321,34 @@
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>Other</t>
+          <t>Supply</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>Low</t>
+          <t>Medium</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t xml:space="preserve">Water is entering the ground floor of the Gampaha </t>
+          <t>Water is entering the ground floor of the Gampaha ...</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>Unknown</t>
+          <t>Gampaha</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>Other</t>
+          <t>Supply</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>Low</t>
+          <t>Medium</t>
         </is>
       </c>
     </row>
@@ -1365,12 +1365,12 @@
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>Other</t>
+          <t>Info</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>Low</t>
+          <t>Medium</t>
         </is>
       </c>
     </row>
@@ -1387,7 +1387,7 @@
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>Other</t>
+          <t>Info</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
@@ -1399,7 +1399,7 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t xml:space="preserve">Helicopter rescue needed for a group of hikers in </t>
+          <t>Helicopter rescue needed for a group of hikers in ...</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
@@ -1409,12 +1409,12 @@
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>Other</t>
+          <t>Rescue</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>Low</t>
+          <t>High</t>
         </is>
       </c>
     </row>
@@ -1426,24 +1426,24 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>Unknown</t>
+          <t>Kandy</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>Other</t>
+          <t>Supply</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>Low</t>
+          <t>Medium</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>Road block at the entrance to the highway. Avoid t</t>
+          <t>Road block at the entrance to the highway. Avoid t...</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
@@ -1453,7 +1453,7 @@
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>Other</t>
+          <t>Info</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
@@ -1475,7 +1475,7 @@
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>Other</t>
+          <t>Info</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
@@ -1497,19 +1497,19 @@
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>Other</t>
+          <t>Rescue</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>Low</t>
+          <t>High</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>The army is distributing food in the affected area</t>
+          <t>The army is distributing food in the affected area...</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
@@ -1519,12 +1519,12 @@
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>Other</t>
+          <t>Supply</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>Low</t>
+          <t>Medium</t>
         </is>
       </c>
     </row>
@@ -1541,7 +1541,7 @@
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>Other</t>
+          <t>Info</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">

</xml_diff>